<commit_message>
docs: update manual test cases and automation table
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\qrius-playwright\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AB94C0F-ECEC-4ED5-9A83-1312A9FC4012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C33F7971-9EDE-44A4-A7A9-E05C0219DB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{59B1DBA9-5E93-44B0-B118-87132858B157}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{59B1DBA9-5E93-44B0-B118-87132858B157}"/>
   </bookViews>
   <sheets>
     <sheet name="Manual test cases" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="160">
   <si>
     <t>S.No</t>
   </si>
@@ -639,6 +639,9 @@
   </si>
   <si>
     <t>users.json</t>
+  </si>
+  <si>
+    <t>Pass</t>
   </si>
 </sst>
 </file>
@@ -1119,7 +1122,7 @@
         <v>21</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>22</v>
+        <v>159</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>23</v>
@@ -1166,7 +1169,7 @@
         <v>30</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>22</v>
+        <v>159</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>23</v>
@@ -1570,8 +1573,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="16.81640625" customWidth="1"/>
-    <col min="3" max="3" width="16.6328125" customWidth="1"/>
-    <col min="4" max="4" width="12.81640625" customWidth="1"/>
+    <col min="3" max="4" width="16.6328125" customWidth="1"/>
     <col min="5" max="5" width="12.54296875" customWidth="1"/>
     <col min="6" max="6" width="16.54296875" customWidth="1"/>
     <col min="7" max="7" width="17.7265625" customWidth="1"/>

</xml_diff>